<commit_message>
Résolution de certains problèmes
</commit_message>
<xml_diff>
--- a/import-enseignants.xlsx
+++ b/import-enseignants.xlsx
@@ -397,7 +397,19 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J46"/>
+  <dimension ref="A1:J64"/>
+  <cols>
+    <col min="1" max="1" width="12.83203125" customWidth="1"/>
+    <col min="2" max="2" width="12.83203125" customWidth="1"/>
+    <col min="3" max="3" width="40.83203125" customWidth="1"/>
+    <col min="4" max="4" width="16.83203125" customWidth="1"/>
+    <col min="5" max="5" width="16.83203125" customWidth="1"/>
+    <col min="6" max="6" width="12.83203125" customWidth="1"/>
+    <col min="7" max="7" width="6.83203125" customWidth="1"/>
+    <col min="8" max="8" width="50.83203125" customWidth="1"/>
+    <col min="9" max="9" width="22.83203125" customWidth="1"/>
+    <col min="10" max="10" width="15.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -433,31 +445,31 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>BIYIHA</v>
+        <v>KAMGA</v>
       </c>
       <c r="B2" t="str">
-        <v>William</v>
+        <v>Emmanuel</v>
       </c>
       <c r="C2" t="str">
-        <v>william.biyiha.teacher020@edu-nexus.cm</v>
+        <v>emmanuel.kamga.teacher001@edu-nexus.cm</v>
       </c>
       <c r="D2" t="str">
-        <v>+237672995600</v>
+        <v>+237670000000</v>
       </c>
       <c r="E2" t="str">
-        <v>ENS-2025-020</v>
+        <v>ENS-2025-001</v>
       </c>
       <c r="F2" t="str">
-        <v>15/11/1972</v>
+        <v>01/01/1965</v>
       </c>
       <c r="G2" t="str">
         <v/>
       </c>
       <c r="H2" t="str">
-        <v>Littérature, Histoire</v>
+        <v>Mathématiques</v>
       </c>
       <c r="I2" t="str">
-        <v>1ère A4-Allemand</v>
+        <v>6e A</v>
       </c>
       <c r="J2" t="str">
         <v/>
@@ -465,31 +477,31 @@
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>MENGA</v>
+        <v>TALLA</v>
       </c>
       <c r="B3" t="str">
-        <v>Noel</v>
+        <v>Sylvain</v>
       </c>
       <c r="C3" t="str">
-        <v>noel.menga.teacher016@edu-nexus.cm</v>
+        <v>sylvain.talla.teacher002@edu-nexus.cm</v>
       </c>
       <c r="D3" t="str">
-        <v>+237672436590</v>
+        <v>+237683337891</v>
       </c>
       <c r="E3" t="str">
-        <v>ENS-2025-016</v>
+        <v>ENS-2025-002</v>
       </c>
       <c r="F3" t="str">
-        <v>26/11/1974</v>
+        <v>12/04/1972</v>
       </c>
       <c r="G3" t="str">
         <v/>
       </c>
       <c r="H3" t="str">
-        <v>Littérature, Mathématiques</v>
+        <v>Mathématiques</v>
       </c>
       <c r="I3" t="str">
-        <v>2nde A4-Chinois</v>
+        <v>5e A</v>
       </c>
       <c r="J3" t="str">
         <v/>
@@ -497,63 +509,63 @@
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>EDZOA</v>
+        <v>NKEMENI</v>
       </c>
       <c r="B4" t="str">
-        <v>Daniel</v>
+        <v>Cédric</v>
       </c>
       <c r="C4" t="str">
-        <v>daniel.edzoa.teacher034@edu-nexus.cm</v>
+        <v>cedric.nkemeni.teacher003@edu-nexus.cm</v>
       </c>
       <c r="D4" t="str">
-        <v>+237670457726</v>
+        <v>+237696675782</v>
       </c>
       <c r="E4" t="str">
-        <v>ENS-2025-034</v>
+        <v>ENS-2025-003</v>
       </c>
       <c r="F4" t="str">
-        <v>25/08/1989</v>
+        <v>23/07/1979</v>
       </c>
       <c r="G4" t="str">
         <v/>
       </c>
       <c r="H4" t="str">
-        <v>Systèmes d'Information, Physique</v>
+        <v>Mathématiques</v>
       </c>
       <c r="I4" t="str">
-        <v>Tle TI</v>
+        <v>4e A</v>
       </c>
       <c r="J4" t="str">
-        <v>TIC</v>
+        <v/>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>ESSONO</v>
+        <v>FOPA</v>
       </c>
       <c r="B5" t="str">
-        <v>Sylvie</v>
+        <v>Romain</v>
       </c>
       <c r="C5" t="str">
-        <v>sylvie.essono.teacher037@edu-nexus.cm</v>
+        <v>romain.fopa.teacher004@edu-nexus.cm</v>
       </c>
       <c r="D5" t="str">
-        <v/>
+        <v>+237681013673</v>
       </c>
       <c r="E5" t="str">
-        <v>ENS-2025-037</v>
+        <v>ENS-2025-004</v>
       </c>
       <c r="F5" t="str">
-        <v/>
+        <v>06/10/1986</v>
       </c>
       <c r="G5" t="str">
         <v/>
       </c>
       <c r="H5" t="str">
-        <v>LV2</v>
+        <v>Mathématiques</v>
       </c>
       <c r="I5" t="str">
-        <v/>
+        <v>3e A</v>
       </c>
       <c r="J5" t="str">
         <v/>
@@ -561,31 +573,31 @@
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>EKANI</v>
+        <v>KOUAM</v>
       </c>
       <c r="B6" t="str">
-        <v>Odile</v>
+        <v>Thierry</v>
       </c>
       <c r="C6" t="str">
-        <v>odile.ekani.teacher029@edu-nexus.cm</v>
+        <v>thierry.kouam.teacher005@edu-nexus.cm</v>
       </c>
       <c r="D6" t="str">
-        <v>+237672178671</v>
+        <v>+237694351564</v>
       </c>
       <c r="E6" t="str">
-        <v>ENS-2025-029</v>
+        <v>ENS-2025-005</v>
       </c>
       <c r="F6" t="str">
-        <v>19/08/1985</v>
+        <v>17/01/1993</v>
       </c>
       <c r="G6" t="str">
         <v/>
       </c>
       <c r="H6" t="str">
-        <v>Philosophie, Géographie, Informatique</v>
+        <v>Mathématiques</v>
       </c>
       <c r="I6" t="str">
-        <v>Tle A4-Arabe</v>
+        <v>2nde C</v>
       </c>
       <c r="J6" t="str">
         <v/>
@@ -593,31 +605,31 @@
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>ENONE</v>
+        <v>MBALLA</v>
       </c>
       <c r="B7" t="str">
-        <v>Toussaint</v>
+        <v>Sophie</v>
       </c>
       <c r="C7" t="str">
-        <v>toussaint.enone.teacher003@edu-nexus.cm</v>
+        <v>sophie.mballa.teacher006@edu-nexus.cm</v>
       </c>
       <c r="D7" t="str">
-        <v>+237675277237</v>
+        <v>+237678689455</v>
       </c>
       <c r="E7" t="str">
-        <v>ENS-2025-003</v>
+        <v>ENS-2025-006</v>
       </c>
       <c r="F7" t="str">
-        <v>20/08/1973</v>
+        <v>28/04/1970</v>
       </c>
       <c r="G7" t="str">
         <v/>
       </c>
       <c r="H7" t="str">
-        <v>Francais, Informatique</v>
+        <v>Français</v>
       </c>
       <c r="I7" t="str">
-        <v>6e C</v>
+        <v>6e B</v>
       </c>
       <c r="J7" t="str">
         <v/>
@@ -625,63 +637,63 @@
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>TSALA</v>
+        <v>ESSOMBA</v>
       </c>
       <c r="B8" t="str">
-        <v>William</v>
+        <v>Christine</v>
       </c>
       <c r="C8" t="str">
-        <v>william.tsala.teacher021@edu-nexus.cm</v>
+        <v>christine.essomba.teacher007@edu-nexus.cm</v>
       </c>
       <c r="D8" t="str">
-        <v>+237674369273</v>
+        <v>+237692027346</v>
       </c>
       <c r="E8" t="str">
-        <v>ENS-2025-021</v>
+        <v>ENS-2025-007</v>
       </c>
       <c r="F8" t="str">
-        <v>23/06/1974</v>
+        <v>11/07/1977</v>
       </c>
       <c r="G8" t="str">
         <v/>
       </c>
       <c r="H8" t="str">
-        <v>Littérature, Histoire, Mathématiques</v>
+        <v>Français</v>
       </c>
       <c r="I8" t="str">
-        <v>1ère A4-Arabe</v>
+        <v>5e B</v>
       </c>
       <c r="J8" t="str">
-        <v>Lettres</v>
+        <v/>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>EBENE</v>
+        <v>ATEBA</v>
       </c>
       <c r="B9" t="str">
-        <v>Josephine</v>
+        <v>Didier</v>
       </c>
       <c r="C9" t="str">
-        <v>josephine.ebene.teacher043@edu-nexus.cm</v>
+        <v>didier.ateba.teacher008@edu-nexus.cm</v>
       </c>
       <c r="D9" t="str">
-        <v/>
+        <v>+237676365237</v>
       </c>
       <c r="E9" t="str">
-        <v>ENS-2025-043</v>
+        <v>ENS-2025-008</v>
       </c>
       <c r="F9" t="str">
-        <v/>
+        <v>22/10/1984</v>
       </c>
       <c r="G9" t="str">
         <v/>
       </c>
       <c r="H9" t="str">
-        <v>Littérature, Langue Française, Français</v>
+        <v>Français</v>
       </c>
       <c r="I9" t="str">
-        <v/>
+        <v>4e B</v>
       </c>
       <c r="J9" t="str">
         <v/>
@@ -689,31 +701,31 @@
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>OWONA</v>
+        <v>NGONO</v>
       </c>
       <c r="B10" t="str">
-        <v>Simon</v>
+        <v>Patrick</v>
       </c>
       <c r="C10" t="str">
-        <v>simon.owona.teacher028@edu-nexus.cm</v>
+        <v>patrick.ngono.teacher009@edu-nexus.cm</v>
       </c>
       <c r="D10" t="str">
-        <v>+237670008861</v>
+        <v>+237689703128</v>
       </c>
       <c r="E10" t="str">
-        <v>ENS-2025-028</v>
+        <v>ENS-2025-009</v>
       </c>
       <c r="F10" t="str">
-        <v>07/08/1976</v>
+        <v>05/01/1991</v>
       </c>
       <c r="G10" t="str">
         <v/>
       </c>
       <c r="H10" t="str">
-        <v>Philosophie, Anglais, Histoire</v>
+        <v>Anglais</v>
       </c>
       <c r="I10" t="str">
-        <v>Tle A4-Allemand</v>
+        <v>6e C</v>
       </c>
       <c r="J10" t="str">
         <v/>
@@ -721,31 +733,31 @@
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>ETOA</v>
+        <v>ABEGA</v>
       </c>
       <c r="B11" t="str">
-        <v>Vincent</v>
+        <v>Laurent</v>
       </c>
       <c r="C11" t="str">
-        <v>vincent.etoa.teacher007@edu-nexus.cm</v>
+        <v>laurent.abega.teacher010@edu-nexus.cm</v>
       </c>
       <c r="D11" t="str">
-        <v>+237676112180</v>
+        <v>+237674041019</v>
       </c>
       <c r="E11" t="str">
-        <v>ENS-2025-007</v>
+        <v>ENS-2025-010</v>
       </c>
       <c r="F11" t="str">
-        <v>02/01/1985</v>
+        <v>16/04/1968</v>
       </c>
       <c r="G11" t="str">
         <v/>
       </c>
       <c r="H11" t="str">
-        <v>Francais, Anglais</v>
+        <v>Anglais</v>
       </c>
       <c r="I11" t="str">
-        <v>4e A</v>
+        <v>5e C</v>
       </c>
       <c r="J11" t="str">
         <v/>
@@ -753,31 +765,31 @@
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>EYEBE</v>
+        <v>FOUDA</v>
       </c>
       <c r="B12" t="str">
-        <v>Anicet</v>
+        <v>Eric</v>
       </c>
       <c r="C12" t="str">
-        <v>anicet.eyebe.teacher040@edu-nexus.cm</v>
+        <v>eric.fouda.teacher011@edu-nexus.cm</v>
       </c>
       <c r="D12" t="str">
-        <v/>
+        <v>+237687378910</v>
       </c>
       <c r="E12" t="str">
-        <v>ENS-2025-040</v>
+        <v>ENS-2025-011</v>
       </c>
       <c r="F12" t="str">
-        <v/>
+        <v>27/07/1975</v>
       </c>
       <c r="G12" t="str">
         <v/>
       </c>
       <c r="H12" t="str">
-        <v>Maintenance et Multimédia, Réseau Internet Sécurité</v>
+        <v>Anglais</v>
       </c>
       <c r="I12" t="str">
-        <v/>
+        <v>4e C</v>
       </c>
       <c r="J12" t="str">
         <v/>
@@ -785,63 +797,63 @@
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>EDZOA</v>
+        <v>ETOUNDI</v>
       </c>
       <c r="B13" t="str">
-        <v>Simon</v>
+        <v>Nicolas</v>
       </c>
       <c r="C13" t="str">
-        <v>simon.edzoa.teacher023@edu-nexus.cm</v>
+        <v>nicolas.etoundi.teacher012@edu-nexus.cm</v>
       </c>
       <c r="D13" t="str">
-        <v>+237675548397</v>
+        <v>+237671716801</v>
       </c>
       <c r="E13" t="str">
-        <v>ENS-2025-023</v>
+        <v>ENS-2025-012</v>
       </c>
       <c r="F13" t="str">
-        <v>26/01/1981</v>
+        <v>10/10/1982</v>
       </c>
       <c r="G13" t="str">
         <v/>
       </c>
       <c r="H13" t="str">
-        <v>Littérature, Géographie</v>
+        <v>Anglais</v>
       </c>
       <c r="I13" t="str">
-        <v>1ère A4-Espagnol</v>
+        <v>3e B</v>
       </c>
       <c r="J13" t="str">
-        <v>EPS</v>
+        <v/>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>SOHAING</v>
+        <v>OWONA</v>
       </c>
       <c r="B14" t="str">
-        <v>Beatrice</v>
+        <v>Marie</v>
       </c>
       <c r="C14" t="str">
-        <v>beatrice.sohaing.teacher017@edu-nexus.cm</v>
+        <v>marie.owona.teacher013@edu-nexus.cm</v>
       </c>
       <c r="D14" t="str">
-        <v>+237671694264</v>
+        <v>+237685054692</v>
       </c>
       <c r="E14" t="str">
-        <v>ENS-2025-017</v>
+        <v>ENS-2025-013</v>
       </c>
       <c r="F14" t="str">
-        <v>25/02/1973</v>
+        <v>21/01/1989</v>
       </c>
       <c r="G14" t="str">
         <v/>
       </c>
       <c r="H14" t="str">
-        <v>Littérature, Mathématiques, Géographie</v>
+        <v>Anglais</v>
       </c>
       <c r="I14" t="str">
-        <v>2nde A4-Espagnol</v>
+        <v>2nde A4-Arabe</v>
       </c>
       <c r="J14" t="str">
         <v/>
@@ -849,31 +861,31 @@
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>TSOPGNI</v>
+        <v>MENGUE</v>
       </c>
       <c r="B15" t="str">
-        <v>Roland</v>
+        <v>Véronique</v>
       </c>
       <c r="C15" t="str">
-        <v>roland.tsopgni.teacher033@edu-nexus.cm</v>
+        <v>veronique.mengue.teacher014@edu-nexus.cm</v>
       </c>
       <c r="D15" t="str">
-        <v>+237675301647</v>
+        <v>+237698392583</v>
       </c>
       <c r="E15" t="str">
-        <v>ENS-2025-033</v>
+        <v>ENS-2025-014</v>
       </c>
       <c r="F15" t="str">
-        <v>23/04/1976</v>
+        <v>04/04/1966</v>
       </c>
       <c r="G15" t="str">
         <v/>
       </c>
       <c r="H15" t="str">
-        <v>Mathématiques, Physique</v>
+        <v>Histoire-Géographie</v>
       </c>
       <c r="I15" t="str">
-        <v>Tle D</v>
+        <v>6e D</v>
       </c>
       <c r="J15" t="str">
         <v/>
@@ -881,63 +893,63 @@
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>MBARGA</v>
+        <v>ASSOUMOU</v>
       </c>
       <c r="B16" t="str">
-        <v>Odile</v>
+        <v>Bernard</v>
       </c>
       <c r="C16" t="str">
-        <v>odile.mbarga.teacher004@edu-nexus.cm</v>
+        <v>bernard.assoumou.teacher015@edu-nexus.cm</v>
       </c>
       <c r="D16" t="str">
-        <v>+237679462272</v>
+        <v>+237682730474</v>
       </c>
       <c r="E16" t="str">
-        <v>ENS-2025-004</v>
+        <v>ENS-2025-015</v>
       </c>
       <c r="F16" t="str">
-        <v>09/10/1989</v>
+        <v>15/07/1973</v>
       </c>
       <c r="G16" t="str">
         <v/>
       </c>
       <c r="H16" t="str">
-        <v>Francais, Histoire, Anglais</v>
+        <v>Histoire-Géographie</v>
       </c>
       <c r="I16" t="str">
-        <v>5e A</v>
+        <v>5e D</v>
       </c>
       <c r="J16" t="str">
-        <v>Arts</v>
+        <v/>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>MVOGO</v>
+        <v>BIDIAS</v>
       </c>
       <c r="B17" t="str">
-        <v>Roland</v>
+        <v>Jean</v>
       </c>
       <c r="C17" t="str">
-        <v>roland.mvogo.teacher008@edu-nexus.cm</v>
+        <v>jean.bidias.teacher016@edu-nexus.cm</v>
       </c>
       <c r="D17" t="str">
-        <v>+237679847324</v>
+        <v>+237696068365</v>
       </c>
       <c r="E17" t="str">
-        <v>ENS-2025-008</v>
+        <v>ENS-2025-016</v>
       </c>
       <c r="F17" t="str">
-        <v>08/07/1976</v>
+        <v>26/10/1980</v>
       </c>
       <c r="G17" t="str">
         <v/>
       </c>
       <c r="H17" t="str">
-        <v>Francais, Physique-Chimie-Technologie</v>
+        <v>Histoire, Géographie</v>
       </c>
       <c r="I17" t="str">
-        <v>4e B</v>
+        <v>4e D</v>
       </c>
       <c r="J17" t="str">
         <v/>
@@ -945,63 +957,63 @@
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>MBOTTO</v>
+        <v>NGANDJUI</v>
       </c>
       <c r="B18" t="str">
-        <v>Ivan</v>
+        <v>Anne</v>
       </c>
       <c r="C18" t="str">
-        <v>ivan.mbotto.teacher027@edu-nexus.cm</v>
+        <v>anne.ngandjui.teacher017@edu-nexus.cm</v>
       </c>
       <c r="D18" t="str">
-        <v>+237671937208</v>
+        <v>+237680406256</v>
       </c>
       <c r="E18" t="str">
-        <v>ENS-2025-027</v>
+        <v>ENS-2025-017</v>
       </c>
       <c r="F18" t="str">
-        <v>13/03/1972</v>
+        <v>09/01/1987</v>
       </c>
       <c r="G18" t="str">
         <v/>
       </c>
       <c r="H18" t="str">
-        <v>Philosophie, Histoire</v>
+        <v>Histoire, Géographie</v>
       </c>
       <c r="I18" t="str">
-        <v>Tle ABI</v>
+        <v>3e C</v>
       </c>
       <c r="J18" t="str">
-        <v>Langues</v>
+        <v/>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>NGONO</v>
+        <v>ONDOUA</v>
       </c>
       <c r="B19" t="str">
-        <v>Nadine</v>
+        <v>Alain</v>
       </c>
       <c r="C19" t="str">
-        <v>nadine.ngono.teacher005@edu-nexus.cm</v>
+        <v>alain.ondoua.teacher018@edu-nexus.cm</v>
       </c>
       <c r="D19" t="str">
-        <v>+237672580309</v>
+        <v>+237693744147</v>
       </c>
       <c r="E19" t="str">
-        <v>ENS-2025-005</v>
+        <v>ENS-2025-018</v>
       </c>
       <c r="F19" t="str">
-        <v>06/04/1977</v>
+        <v>20/04/1994</v>
       </c>
       <c r="G19" t="str">
         <v/>
       </c>
       <c r="H19" t="str">
-        <v>Francais, EPS, Informatique</v>
+        <v>Physique-Chimie, Physique-Chimie-Technologie</v>
       </c>
       <c r="I19" t="str">
-        <v>5e B</v>
+        <v>3e D</v>
       </c>
       <c r="J19" t="str">
         <v/>
@@ -1009,31 +1021,31 @@
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>NKOTTI</v>
+        <v>NGOUNOU</v>
       </c>
       <c r="B20" t="str">
-        <v>Pierre</v>
+        <v>Philippe</v>
       </c>
       <c r="C20" t="str">
-        <v>pierre.nkotti.teacher042@edu-nexus.cm</v>
+        <v>philippe.ngounou.teacher019@edu-nexus.cm</v>
       </c>
       <c r="D20" t="str">
-        <v/>
+        <v>+237678082038</v>
       </c>
       <c r="E20" t="str">
-        <v>ENS-2025-042</v>
+        <v>ENS-2025-019</v>
       </c>
       <c r="F20" t="str">
-        <v/>
+        <v>03/07/1971</v>
       </c>
       <c r="G20" t="str">
         <v/>
       </c>
       <c r="H20" t="str">
-        <v>SVTEEHB, Physique-Chimie-Technologie</v>
+        <v>Physique, Chimie</v>
       </c>
       <c r="I20" t="str">
-        <v/>
+        <v>1ère C</v>
       </c>
       <c r="J20" t="str">
         <v/>
@@ -1041,31 +1053,31 @@
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>ZOA</v>
+        <v>DONFACK</v>
       </c>
       <c r="B21" t="str">
-        <v>Toussaint</v>
+        <v>Hélène</v>
       </c>
       <c r="C21" t="str">
-        <v>toussaint.zoa.teacher024@edu-nexus.cm</v>
+        <v>helene.donfack.teacher020@edu-nexus.cm</v>
       </c>
       <c r="D21" t="str">
-        <v>+237678754502</v>
+        <v>+237691419929</v>
       </c>
       <c r="E21" t="str">
-        <v>ENS-2025-024</v>
+        <v>ENS-2025-020</v>
       </c>
       <c r="F21" t="str">
-        <v>07/06/1986</v>
+        <v>14/10/1978</v>
       </c>
       <c r="G21" t="str">
         <v/>
       </c>
       <c r="H21" t="str">
-        <v>Physique, Anglais, SVTEEHB</v>
+        <v>Physique, Chimie</v>
       </c>
       <c r="I21" t="str">
-        <v>1ère C</v>
+        <v>Tle C</v>
       </c>
       <c r="J21" t="str">
         <v/>
@@ -1073,31 +1085,31 @@
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>SOHAING</v>
+        <v>TCHOUGANG</v>
       </c>
       <c r="B22" t="str">
-        <v>Daniel</v>
+        <v>Michel</v>
       </c>
       <c r="C22" t="str">
-        <v>daniel.sohaing.teacher011@edu-nexus.cm</v>
+        <v>michel.tchougang.teacher021@edu-nexus.cm</v>
       </c>
       <c r="D22" t="str">
-        <v>+237673846654</v>
+        <v>+237675757820</v>
       </c>
       <c r="E22" t="str">
-        <v>ENS-2025-011</v>
+        <v>ENS-2025-021</v>
       </c>
       <c r="F22" t="str">
-        <v>17/10/1976</v>
+        <v>25/01/1985</v>
       </c>
       <c r="G22" t="str">
         <v/>
       </c>
       <c r="H22" t="str">
-        <v>Francais, LV2, Physique-Chimie-Technologie</v>
+        <v>SVTEEHB, SVT</v>
       </c>
       <c r="I22" t="str">
-        <v>3e B</v>
+        <v>1ère D</v>
       </c>
       <c r="J22" t="str">
         <v/>
@@ -1105,31 +1117,31 @@
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>TSOPGNI</v>
+        <v>SAMBA</v>
       </c>
       <c r="B23" t="str">
-        <v>Jules</v>
+        <v>Isabelle</v>
       </c>
       <c r="C23" t="str">
-        <v>jules.tsopgni.teacher013@edu-nexus.cm</v>
+        <v>isabelle.samba.teacher022@edu-nexus.cm</v>
       </c>
       <c r="D23" t="str">
-        <v>+237676352517</v>
+        <v>+237689095711</v>
       </c>
       <c r="E23" t="str">
-        <v>ENS-2025-013</v>
+        <v>ENS-2025-022</v>
       </c>
       <c r="F23" t="str">
-        <v>22/11/1971</v>
+        <v>08/04/1992</v>
       </c>
       <c r="G23" t="str">
         <v/>
       </c>
       <c r="H23" t="str">
-        <v>Intensive English, Informatique, Géographie</v>
+        <v>SVTEEHB, SVT</v>
       </c>
       <c r="I23" t="str">
-        <v>2nde ABI</v>
+        <v>Tle D</v>
       </c>
       <c r="J23" t="str">
         <v/>
@@ -1137,31 +1149,31 @@
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>NGONO</v>
+        <v>WAMBA</v>
       </c>
       <c r="B24" t="str">
-        <v>Marguerite</v>
+        <v>Carole</v>
       </c>
       <c r="C24" t="str">
-        <v>marguerite.ngono.teacher030@edu-nexus.cm</v>
+        <v>carole.wamba.teacher023@edu-nexus.cm</v>
       </c>
       <c r="D24" t="str">
-        <v>+237672811400</v>
+        <v>+237673433602</v>
       </c>
       <c r="E24" t="str">
-        <v>ENS-2025-030</v>
+        <v>ENS-2025-023</v>
       </c>
       <c r="F24" t="str">
-        <v>26/09/1985</v>
+        <v>19/07/1969</v>
       </c>
       <c r="G24" t="str">
         <v/>
       </c>
       <c r="H24" t="str">
-        <v>Philosophie, Éducation Artistique</v>
+        <v>EPS</v>
       </c>
       <c r="I24" t="str">
-        <v>Tle A4-Chinois</v>
+        <v>2nde A4-Allemand</v>
       </c>
       <c r="J24" t="str">
         <v/>
@@ -1169,31 +1181,31 @@
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>MIMBOE</v>
+        <v>DIFFO</v>
       </c>
       <c r="B25" t="str">
-        <v>Noel</v>
+        <v>Luc</v>
       </c>
       <c r="C25" t="str">
-        <v>noel.mimboe.teacher010@edu-nexus.cm</v>
+        <v>luc.diffo.teacher024@edu-nexus.cm</v>
       </c>
       <c r="D25" t="str">
-        <v>+237672253683</v>
+        <v>+237686771493</v>
       </c>
       <c r="E25" t="str">
-        <v>ENS-2025-010</v>
+        <v>ENS-2025-024</v>
       </c>
       <c r="F25" t="str">
-        <v>17/09/1974</v>
+        <v>02/10/1976</v>
       </c>
       <c r="G25" t="str">
         <v/>
       </c>
       <c r="H25" t="str">
-        <v>Francais, LV2, EPS</v>
+        <v>EPS</v>
       </c>
       <c r="I25" t="str">
-        <v>3e A</v>
+        <v>2nde A4-Espagnol</v>
       </c>
       <c r="J25" t="str">
         <v/>
@@ -1201,31 +1213,31 @@
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>EBENE</v>
+        <v>MONTHE</v>
       </c>
       <c r="B26" t="str">
-        <v>Flavie</v>
+        <v>Stéphane</v>
       </c>
       <c r="C26" t="str">
-        <v>flavie.ebene.teacher031@edu-nexus.cm</v>
+        <v>stephane.monthe.teacher025@edu-nexus.cm</v>
       </c>
       <c r="D26" t="str">
-        <v>+237676896234</v>
+        <v>+237671109384</v>
       </c>
       <c r="E26" t="str">
-        <v>ENS-2025-031</v>
+        <v>ENS-2025-025</v>
       </c>
       <c r="F26" t="str">
-        <v>24/08/1975</v>
+        <v>13/01/1983</v>
       </c>
       <c r="G26" t="str">
         <v/>
       </c>
       <c r="H26" t="str">
-        <v>Philosophie, Éducation Artistique, Anglais</v>
+        <v>EPS</v>
       </c>
       <c r="I26" t="str">
-        <v>Tle A4-Espagnol</v>
+        <v>2nde D</v>
       </c>
       <c r="J26" t="str">
         <v/>
@@ -1233,31 +1245,31 @@
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>ZOA</v>
+        <v>ZANG</v>
       </c>
       <c r="B27" t="str">
-        <v>Nadine</v>
+        <v>Pauline</v>
       </c>
       <c r="C27" t="str">
-        <v>nadine.zoa.teacher015@edu-nexus.cm</v>
+        <v>pauline.zang.teacher026@edu-nexus.cm</v>
       </c>
       <c r="D27" t="str">
-        <v>+237672982765</v>
+        <v>+237684447275</v>
       </c>
       <c r="E27" t="str">
-        <v>ENS-2025-015</v>
+        <v>ENS-2025-026</v>
       </c>
       <c r="F27" t="str">
-        <v>02/03/1979</v>
+        <v>24/04/1990</v>
       </c>
       <c r="G27" t="str">
         <v/>
       </c>
       <c r="H27" t="str">
-        <v>Littérature, Éducation Artistique</v>
+        <v>Littérature, Langue Française</v>
       </c>
       <c r="I27" t="str">
-        <v>2nde A4-Arabe</v>
+        <v>1ère A4-Allemand</v>
       </c>
       <c r="J27" t="str">
         <v/>
@@ -1265,31 +1277,31 @@
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>MVOGO</v>
+        <v>BIYIHA</v>
       </c>
       <c r="B28" t="str">
-        <v>Therese</v>
+        <v>William</v>
       </c>
       <c r="C28" t="str">
-        <v>therese.mvogo.teacher041@edu-nexus.cm</v>
+        <v>william.biyiha.teacher027@edu-nexus.cm</v>
       </c>
       <c r="D28" t="str">
-        <v/>
+        <v>+237697785166</v>
       </c>
       <c r="E28" t="str">
-        <v>ENS-2025-041</v>
+        <v>ENS-2025-027</v>
       </c>
       <c r="F28" t="str">
-        <v/>
+        <v>07/07/1967</v>
       </c>
       <c r="G28" t="str">
         <v/>
       </c>
       <c r="H28" t="str">
-        <v>Physique, Chimie, Sciences</v>
+        <v>Littérature, Langue Française</v>
       </c>
       <c r="I28" t="str">
-        <v/>
+        <v>1ère A4-Arabe</v>
       </c>
       <c r="J28" t="str">
         <v/>
@@ -1297,31 +1309,31 @@
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>EDZOA</v>
+        <v>NGUELE</v>
       </c>
       <c r="B29" t="str">
-        <v>Rene</v>
+        <v>Carole</v>
       </c>
       <c r="C29" t="str">
-        <v>rene.edzoa.teacher044@edu-nexus.cm</v>
+        <v>carole.nguele.teacher028@edu-nexus.cm</v>
       </c>
       <c r="D29" t="str">
-        <v/>
+        <v>+237682123057</v>
       </c>
       <c r="E29" t="str">
-        <v>ENS-2025-044</v>
+        <v>ENS-2025-028</v>
       </c>
       <c r="F29" t="str">
-        <v/>
+        <v>18/10/1974</v>
       </c>
       <c r="G29" t="str">
         <v/>
       </c>
       <c r="H29" t="str">
-        <v>Philosophie, Lettres classiques (Latin/Grec)</v>
+        <v>Littérature, Langue Française</v>
       </c>
       <c r="I29" t="str">
-        <v/>
+        <v>1ère A4-Chinois</v>
       </c>
       <c r="J29" t="str">
         <v/>
@@ -1329,31 +1341,31 @@
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>ONDOUA</v>
+        <v>MVOMO</v>
       </c>
       <c r="B30" t="str">
-        <v>Jose</v>
+        <v>Antoine</v>
       </c>
       <c r="C30" t="str">
-        <v>jose.ondoua.teacher038@edu-nexus.cm</v>
+        <v>antoine.mvomo.teacher029@edu-nexus.cm</v>
       </c>
       <c r="D30" t="str">
-        <v/>
+        <v>+237695460948</v>
       </c>
       <c r="E30" t="str">
-        <v>ENS-2025-038</v>
+        <v>ENS-2025-029</v>
       </c>
       <c r="F30" t="str">
-        <v/>
+        <v>01/01/1981</v>
       </c>
       <c r="G30" t="str">
         <v/>
       </c>
       <c r="H30" t="str">
-        <v>LV2</v>
+        <v>Littérature, Langue Française</v>
       </c>
       <c r="I30" t="str">
-        <v/>
+        <v>1ère A4-Espagnol</v>
       </c>
       <c r="J30" t="str">
         <v/>
@@ -1361,31 +1373,31 @@
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>NNANGA</v>
+        <v>NGAMENI</v>
       </c>
       <c r="B31" t="str">
-        <v>Simon</v>
+        <v>Robert</v>
       </c>
       <c r="C31" t="str">
-        <v>simon.nnanga.teacher002@edu-nexus.cm</v>
+        <v>robert.ngameni.teacher030@edu-nexus.cm</v>
       </c>
       <c r="D31" t="str">
-        <v>+237677522968</v>
+        <v>+237679798839</v>
       </c>
       <c r="E31" t="str">
-        <v>ENS-2025-002</v>
+        <v>ENS-2025-030</v>
       </c>
       <c r="F31" t="str">
-        <v>09/03/1977</v>
+        <v>12/04/1988</v>
       </c>
       <c r="G31" t="str">
         <v/>
       </c>
       <c r="H31" t="str">
-        <v>Francais, Informatique</v>
+        <v>Allemand</v>
       </c>
       <c r="I31" t="str">
-        <v>6e B</v>
+        <v>Tle A4-Allemand</v>
       </c>
       <c r="J31" t="str">
         <v/>
@@ -1393,31 +1405,31 @@
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>ETOA</v>
+        <v>KENFACK</v>
       </c>
       <c r="B32" t="str">
-        <v>Fernand</v>
+        <v>Julie</v>
       </c>
       <c r="C32" t="str">
-        <v>fernand.etoa.teacher018@edu-nexus.cm</v>
+        <v>julie.kenfack.teacher031@edu-nexus.cm</v>
       </c>
       <c r="D32" t="str">
-        <v>+237671571505</v>
+        <v>+237693136730</v>
       </c>
       <c r="E32" t="str">
-        <v>ENS-2025-018</v>
+        <v>ENS-2025-031</v>
       </c>
       <c r="F32" t="str">
-        <v>07/09/1975</v>
+        <v>23/07/1965</v>
       </c>
       <c r="G32" t="str">
         <v/>
       </c>
       <c r="H32" t="str">
-        <v>Mathématiques, Informatique, Physique</v>
+        <v>Espagnol</v>
       </c>
       <c r="I32" t="str">
-        <v>2nde C</v>
+        <v>Tle A4-Espagnol</v>
       </c>
       <c r="J32" t="str">
         <v/>
@@ -1425,31 +1437,31 @@
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>MIMBOE</v>
+        <v>BELIBI</v>
       </c>
       <c r="B33" t="str">
-        <v>Marcelle</v>
+        <v>Baptiste</v>
       </c>
       <c r="C33" t="str">
-        <v>marcelle.mimboe.teacher035@edu-nexus.cm</v>
+        <v>baptiste.belibi.teacher032@edu-nexus.cm</v>
       </c>
       <c r="D33" t="str">
-        <v/>
+        <v>+237677474621</v>
       </c>
       <c r="E33" t="str">
-        <v>ENS-2025-035</v>
+        <v>ENS-2025-032</v>
       </c>
       <c r="F33" t="str">
-        <v/>
+        <v>06/10/1972</v>
       </c>
       <c r="G33" t="str">
         <v/>
       </c>
       <c r="H33" t="str">
-        <v>LV2</v>
+        <v>Arabe</v>
       </c>
       <c r="I33" t="str">
-        <v/>
+        <v>Tle A4-Arabe</v>
       </c>
       <c r="J33" t="str">
         <v/>
@@ -1457,63 +1469,63 @@
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>ZOGO</v>
+        <v>MANGA</v>
       </c>
       <c r="B34" t="str">
-        <v>Daniel</v>
+        <v>Thomas</v>
       </c>
       <c r="C34" t="str">
-        <v>daniel.zogo.teacher022@edu-nexus.cm</v>
+        <v>thomas.manga.teacher033@edu-nexus.cm</v>
       </c>
       <c r="D34" t="str">
-        <v>+237679064242</v>
+        <v>+237690812512</v>
       </c>
       <c r="E34" t="str">
-        <v>ENS-2025-022</v>
+        <v>ENS-2025-033</v>
       </c>
       <c r="F34" t="str">
-        <v>09/08/1989</v>
+        <v>17/01/1979</v>
       </c>
       <c r="G34" t="str">
         <v/>
       </c>
       <c r="H34" t="str">
-        <v>Littérature, Anglais, Histoire</v>
+        <v>Chinois</v>
       </c>
       <c r="I34" t="str">
-        <v>1ère A4-Chinois</v>
+        <v>Tle A4-Chinois</v>
       </c>
       <c r="J34" t="str">
-        <v>HistoireGeo</v>
+        <v/>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>MVOGO</v>
+        <v>ETOGA</v>
       </c>
       <c r="B35" t="str">
-        <v>Daniel</v>
+        <v>François</v>
       </c>
       <c r="C35" t="str">
-        <v>daniel.mvogo.teacher025@edu-nexus.cm</v>
+        <v>francois.etoga.teacher034@edu-nexus.cm</v>
       </c>
       <c r="D35" t="str">
-        <v>+237670779064</v>
+        <v>+237675150403</v>
       </c>
       <c r="E35" t="str">
-        <v>ENS-2025-025</v>
+        <v>ENS-2025-034</v>
       </c>
       <c r="F35" t="str">
-        <v>13/12/1978</v>
+        <v>28/04/1986</v>
       </c>
       <c r="G35" t="str">
         <v/>
       </c>
       <c r="H35" t="str">
-        <v>SVTEEHB, Chimie, Anglais</v>
+        <v>Philosophie, Éducation à la Citoyenneté et à la Morale</v>
       </c>
       <c r="I35" t="str">
-        <v>1ère D</v>
+        <v>Tle TI</v>
       </c>
       <c r="J35" t="str">
         <v/>
@@ -1521,31 +1533,31 @@
     </row>
     <row r="36">
       <c r="A36" t="str">
-        <v>NOMO</v>
+        <v>NGUEMBI</v>
       </c>
       <c r="B36" t="str">
-        <v>Vincent</v>
+        <v>Sylvie</v>
       </c>
       <c r="C36" t="str">
-        <v>vincent.nomo.teacher019@edu-nexus.cm</v>
+        <v>sylvie.nguembi.teacher035@edu-nexus.cm</v>
       </c>
       <c r="D36" t="str">
-        <v>+237676313633</v>
+        <v>+237688488294</v>
       </c>
       <c r="E36" t="str">
-        <v>ENS-2025-019</v>
+        <v>ENS-2025-035</v>
       </c>
       <c r="F36" t="str">
-        <v>13/11/1987</v>
+        <v>11/07/1993</v>
       </c>
       <c r="G36" t="str">
         <v/>
       </c>
       <c r="H36" t="str">
-        <v>Intensive English, Histoire, Géographie</v>
+        <v>Philosophie, Éducation à la Citoyenneté et à la Morale</v>
       </c>
       <c r="I36" t="str">
-        <v>1ère ABI</v>
+        <v>1ère TI</v>
       </c>
       <c r="J36" t="str">
         <v/>
@@ -1553,31 +1565,31 @@
     </row>
     <row r="37">
       <c r="A37" t="str">
-        <v>ESSONO</v>
+        <v>EDZOA</v>
       </c>
       <c r="B37" t="str">
-        <v>Pascal</v>
+        <v>Daniel</v>
       </c>
       <c r="C37" t="str">
-        <v>pascal.essono.teacher026@edu-nexus.cm</v>
+        <v>daniel.edzoa.teacher036@edu-nexus.cm</v>
       </c>
       <c r="D37" t="str">
-        <v>+237679559684</v>
+        <v>+237672826185</v>
       </c>
       <c r="E37" t="str">
-        <v>ENS-2025-026</v>
+        <v>ENS-2025-036</v>
       </c>
       <c r="F37" t="str">
-        <v>22/03/1984</v>
+        <v>22/10/1970</v>
       </c>
       <c r="G37" t="str">
         <v/>
       </c>
       <c r="H37" t="str">
-        <v>Algorithmique-Programmation, Anglais</v>
+        <v>Informatique, Algorithmique-Programmation</v>
       </c>
       <c r="I37" t="str">
-        <v>1ère TI</v>
+        <v>2nde A4-Chinois</v>
       </c>
       <c r="J37" t="str">
         <v/>
@@ -1585,28 +1597,28 @@
     </row>
     <row r="38">
       <c r="A38" t="str">
-        <v>ZAMBO</v>
+        <v>TEUKAM</v>
       </c>
       <c r="B38" t="str">
-        <v>Marthe</v>
+        <v>Gilles</v>
       </c>
       <c r="C38" t="str">
-        <v>marthe.zambo.teacher045@edu-nexus.cm</v>
+        <v>gilles.teukam.teacher037@edu-nexus.cm</v>
       </c>
       <c r="D38" t="str">
-        <v/>
+        <v>+237686164076</v>
       </c>
       <c r="E38" t="str">
-        <v>ENS-2025-045</v>
+        <v>ENS-2025-037</v>
       </c>
       <c r="F38" t="str">
-        <v/>
+        <v>05/01/1977</v>
       </c>
       <c r="G38" t="str">
         <v/>
       </c>
       <c r="H38" t="str">
-        <v>Histoire, Géographie, Éducation à la Citoyenneté et à la Morale</v>
+        <v>Maintenance et Multimédia, Réseau Internet Sécurité, Programmation</v>
       </c>
       <c r="I38" t="str">
         <v/>
@@ -1617,63 +1629,63 @@
     </row>
     <row r="39">
       <c r="A39" t="str">
-        <v>ZOA</v>
+        <v>NGUEFACK</v>
       </c>
       <c r="B39" t="str">
-        <v>Yolande</v>
+        <v>Alexandre</v>
       </c>
       <c r="C39" t="str">
-        <v>yolande.zoa.teacher009@edu-nexus.cm</v>
+        <v>alexandre.nguefack.teacher038@edu-nexus.cm</v>
       </c>
       <c r="D39" t="str">
-        <v>+237676171028</v>
+        <v>+237670501967</v>
       </c>
       <c r="E39" t="str">
-        <v>ENS-2025-009</v>
+        <v>ENS-2025-038</v>
       </c>
       <c r="F39" t="str">
-        <v>13/03/1976</v>
+        <v>16/04/1984</v>
       </c>
       <c r="G39" t="str">
         <v/>
       </c>
       <c r="H39" t="str">
-        <v>Francais, Anglais, Histoire</v>
+        <v>Systèmes d'Information, Informatique</v>
       </c>
       <c r="I39" t="str">
-        <v>4e C</v>
+        <v/>
       </c>
       <c r="J39" t="str">
-        <v>Sciences</v>
+        <v/>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="str">
-        <v>MEKONGO</v>
+        <v>MVONDO</v>
       </c>
       <c r="B40" t="str">
-        <v>Boris</v>
+        <v>Pierre</v>
       </c>
       <c r="C40" t="str">
-        <v>boris.mekongo.teacher032@edu-nexus.cm</v>
+        <v>pierre.mvondo.teacher039@edu-nexus.cm</v>
       </c>
       <c r="D40" t="str">
-        <v>+237678626501</v>
+        <v>+237683839858</v>
       </c>
       <c r="E40" t="str">
-        <v>ENS-2025-032</v>
+        <v>ENS-2025-039</v>
       </c>
       <c r="F40" t="str">
-        <v>05/02/1984</v>
+        <v>27/07/1991</v>
       </c>
       <c r="G40" t="str">
         <v/>
       </c>
       <c r="H40" t="str">
-        <v>Mathématiques, Informatique, SVTEEHB</v>
+        <v>Mathématiques</v>
       </c>
       <c r="I40" t="str">
-        <v>Tle C</v>
+        <v/>
       </c>
       <c r="J40" t="str">
         <v/>
@@ -1681,31 +1693,31 @@
     </row>
     <row r="41">
       <c r="A41" t="str">
-        <v>ZOGO</v>
+        <v>NGAH</v>
       </c>
       <c r="B41" t="str">
-        <v>Simon</v>
+        <v>Rachel</v>
       </c>
       <c r="C41" t="str">
-        <v>simon.zogo.teacher006@edu-nexus.cm</v>
+        <v>rachel.ngah.teacher040@edu-nexus.cm</v>
       </c>
       <c r="D41" t="str">
-        <v>+237674720287</v>
+        <v>+237697177749</v>
       </c>
       <c r="E41" t="str">
-        <v>ENS-2025-006</v>
+        <v>ENS-2025-040</v>
       </c>
       <c r="F41" t="str">
-        <v>01/12/1978</v>
+        <v>10/10/1968</v>
       </c>
       <c r="G41" t="str">
         <v/>
       </c>
       <c r="H41" t="str">
-        <v>Francais, EPS, Histoire</v>
+        <v>Sciences, SVT</v>
       </c>
       <c r="I41" t="str">
-        <v>5e C</v>
+        <v/>
       </c>
       <c r="J41" t="str">
         <v/>
@@ -1713,28 +1725,28 @@
     </row>
     <row r="42">
       <c r="A42" t="str">
-        <v>TCHINDA</v>
+        <v>ATANGANA</v>
       </c>
       <c r="B42" t="str">
-        <v>Gerard</v>
+        <v>Henri</v>
       </c>
       <c r="C42" t="str">
-        <v>gerard.tchinda.teacher036@edu-nexus.cm</v>
+        <v>henri.atangana.teacher041@edu-nexus.cm</v>
       </c>
       <c r="D42" t="str">
-        <v/>
+        <v>+237681515640</v>
       </c>
       <c r="E42" t="str">
-        <v>ENS-2025-036</v>
+        <v>ENS-2025-041</v>
       </c>
       <c r="F42" t="str">
-        <v/>
+        <v>21/01/1975</v>
       </c>
       <c r="G42" t="str">
         <v/>
       </c>
       <c r="H42" t="str">
-        <v>LV2</v>
+        <v>Éducation à la Citoyenneté et à la Morale, Cultures Nationales, Langues Nationales</v>
       </c>
       <c r="I42" t="str">
         <v/>
@@ -1745,28 +1757,28 @@
     </row>
     <row r="43">
       <c r="A43" t="str">
-        <v>TSALA</v>
+        <v>MONKAM</v>
       </c>
       <c r="B43" t="str">
-        <v>Luc</v>
+        <v>Carine</v>
       </c>
       <c r="C43" t="str">
-        <v>luc.tsala.teacher039@edu-nexus.cm</v>
+        <v>carine.monkam.teacher042@edu-nexus.cm</v>
       </c>
       <c r="D43" t="str">
-        <v/>
+        <v>+237694853531</v>
       </c>
       <c r="E43" t="str">
-        <v>ENS-2025-039</v>
+        <v>ENS-2025-042</v>
       </c>
       <c r="F43" t="str">
-        <v/>
+        <v>04/04/1982</v>
       </c>
       <c r="G43" t="str">
         <v/>
       </c>
       <c r="H43" t="str">
-        <v>Algorithmique-Programmation, Systèmes d'Information, Programmation</v>
+        <v>Travail Manuel, Éducation Artistique, Éducation Artistique et Culturelle</v>
       </c>
       <c r="I43" t="str">
         <v/>
@@ -1777,31 +1789,31 @@
     </row>
     <row r="44">
       <c r="A44" t="str">
-        <v>TCHOUALA</v>
+        <v>NTOUBA</v>
       </c>
       <c r="B44" t="str">
-        <v>Oscar</v>
+        <v>Marc</v>
       </c>
       <c r="C44" t="str">
-        <v>oscar.tchouala.teacher001@edu-nexus.cm</v>
+        <v>marc.ntouba.teacher043@edu-nexus.cm</v>
       </c>
       <c r="D44" t="str">
-        <v>+237679989385</v>
+        <v>+237679191422</v>
       </c>
       <c r="E44" t="str">
-        <v>ENS-2025-001</v>
+        <v>ENS-2025-043</v>
       </c>
       <c r="F44" t="str">
-        <v>15/12/1983</v>
+        <v>15/07/1989</v>
       </c>
       <c r="G44" t="str">
         <v/>
       </c>
       <c r="H44" t="str">
-        <v>Francais, Informatique, Histoire</v>
+        <v>Philosophie</v>
       </c>
       <c r="I44" t="str">
-        <v>6e A</v>
+        <v/>
       </c>
       <c r="J44" t="str">
         <v/>
@@ -1809,31 +1821,31 @@
     </row>
     <row r="45">
       <c r="A45" t="str">
-        <v>MVOGO</v>
+        <v>DIFFO</v>
       </c>
       <c r="B45" t="str">
-        <v>Odile</v>
+        <v>Justine</v>
       </c>
       <c r="C45" t="str">
-        <v>odile.mvogo.teacher014@edu-nexus.cm</v>
+        <v>justine.diffo.teacher044@edu-nexus.cm</v>
       </c>
       <c r="D45" t="str">
-        <v>+237678587664</v>
+        <v>+237692529313</v>
       </c>
       <c r="E45" t="str">
-        <v>ENS-2025-014</v>
+        <v>ENS-2025-044</v>
       </c>
       <c r="F45" t="str">
-        <v>17/03/1984</v>
+        <v>26/10/1966</v>
       </c>
       <c r="G45" t="str">
         <v/>
       </c>
       <c r="H45" t="str">
-        <v>Littérature, Informatique, Histoire</v>
+        <v>Français, Langue Française</v>
       </c>
       <c r="I45" t="str">
-        <v>2nde A4-Allemand</v>
+        <v/>
       </c>
       <c r="J45" t="str">
         <v/>
@@ -1841,39 +1853,615 @@
     </row>
     <row r="46">
       <c r="A46" t="str">
-        <v>TCHOFFO</v>
+        <v>KETCHEMEN</v>
       </c>
       <c r="B46" t="str">
-        <v>Marguerite</v>
+        <v>Paul</v>
       </c>
       <c r="C46" t="str">
-        <v>marguerite.tchoffo.teacher012@edu-nexus.cm</v>
+        <v>paul.ketchemen.teacher045@edu-nexus.cm</v>
       </c>
       <c r="D46" t="str">
-        <v>+237677729175</v>
+        <v>+237676867204</v>
       </c>
       <c r="E46" t="str">
-        <v>ENS-2025-012</v>
+        <v>ENS-2025-045</v>
       </c>
       <c r="F46" t="str">
-        <v>01/04/1983</v>
+        <v>09/01/1973</v>
       </c>
       <c r="G46" t="str">
         <v/>
       </c>
       <c r="H46" t="str">
-        <v>Francais, Mathématiques</v>
+        <v>Histoire, Géographie</v>
       </c>
       <c r="I46" t="str">
-        <v>3e C</v>
+        <v/>
       </c>
       <c r="J46" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="str">
+        <v>DJOMKAM</v>
+      </c>
+      <c r="B47" t="str">
+        <v>Beatrice</v>
+      </c>
+      <c r="C47" t="str">
+        <v>beatrice.djomkam.teacher046@edu-nexus.cm</v>
+      </c>
+      <c r="D47" t="str">
+        <v>+237690205095</v>
+      </c>
+      <c r="E47" t="str">
+        <v>ENS-2025-046</v>
+      </c>
+      <c r="F47" t="str">
+        <v>20/04/1980</v>
+      </c>
+      <c r="G47" t="str">
+        <v/>
+      </c>
+      <c r="H47" t="str">
+        <v>Sciences, Éducation Artistique, Éducation Artistique et Culturelle</v>
+      </c>
+      <c r="I47" t="str">
+        <v/>
+      </c>
+      <c r="J47" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="str">
+        <v>BELLA</v>
+      </c>
+      <c r="B48" t="str">
+        <v>Joseph</v>
+      </c>
+      <c r="C48" t="str">
+        <v>joseph.bella.teacher047@edu-nexus.cm</v>
+      </c>
+      <c r="D48" t="str">
+        <v>+237674542986</v>
+      </c>
+      <c r="E48" t="str">
+        <v>ENS-2025-047</v>
+      </c>
+      <c r="F48" t="str">
+        <v>03/07/1987</v>
+      </c>
+      <c r="G48" t="str">
+        <v/>
+      </c>
+      <c r="H48" t="str">
+        <v>Mathématiques</v>
+      </c>
+      <c r="I48" t="str">
+        <v/>
+      </c>
+      <c r="J48" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="str">
+        <v>NKODO</v>
+      </c>
+      <c r="B49" t="str">
+        <v>Rose</v>
+      </c>
+      <c r="C49" t="str">
+        <v>rose.nkodo.teacher048@edu-nexus.cm</v>
+      </c>
+      <c r="D49" t="str">
+        <v>+237687880877</v>
+      </c>
+      <c r="E49" t="str">
+        <v>ENS-2025-048</v>
+      </c>
+      <c r="F49" t="str">
+        <v>14/10/1994</v>
+      </c>
+      <c r="G49" t="str">
+        <v/>
+      </c>
+      <c r="H49" t="str">
+        <v>Mathématiques</v>
+      </c>
+      <c r="I49" t="str">
+        <v/>
+      </c>
+      <c r="J49" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="str">
+        <v>AMOUGOU</v>
+      </c>
+      <c r="B50" t="str">
+        <v>Théodore</v>
+      </c>
+      <c r="C50" t="str">
+        <v>theodore.amougou.teacher049@edu-nexus.cm</v>
+      </c>
+      <c r="D50" t="str">
+        <v>+237672218768</v>
+      </c>
+      <c r="E50" t="str">
+        <v>ENS-2025-049</v>
+      </c>
+      <c r="F50" t="str">
+        <v>25/01/1971</v>
+      </c>
+      <c r="G50" t="str">
+        <v/>
+      </c>
+      <c r="H50" t="str">
+        <v>Mathématiques</v>
+      </c>
+      <c r="I50" t="str">
+        <v/>
+      </c>
+      <c r="J50" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="str">
+        <v>ONDOA</v>
+      </c>
+      <c r="B51" t="str">
+        <v>Patricia</v>
+      </c>
+      <c r="C51" t="str">
+        <v>patricia.ondoa.teacher050@edu-nexus.cm</v>
+      </c>
+      <c r="D51" t="str">
+        <v>+237685556659</v>
+      </c>
+      <c r="E51" t="str">
+        <v>ENS-2025-050</v>
+      </c>
+      <c r="F51" t="str">
+        <v>08/04/1978</v>
+      </c>
+      <c r="G51" t="str">
+        <v/>
+      </c>
+      <c r="H51" t="str">
+        <v>Français, Langue Française</v>
+      </c>
+      <c r="I51" t="str">
+        <v/>
+      </c>
+      <c r="J51" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="str">
+        <v>FEUDJIO</v>
+      </c>
+      <c r="B52" t="str">
+        <v>Jean-Pierre</v>
+      </c>
+      <c r="C52" t="str">
+        <v>jeanpierre.feudjio.teacher051@edu-nexus.cm</v>
+      </c>
+      <c r="D52" t="str">
+        <v>+237698894550</v>
+      </c>
+      <c r="E52" t="str">
+        <v>ENS-2025-051</v>
+      </c>
+      <c r="F52" t="str">
+        <v>19/07/1985</v>
+      </c>
+      <c r="G52" t="str">
+        <v/>
+      </c>
+      <c r="H52" t="str">
+        <v>Français, Langue Française</v>
+      </c>
+      <c r="I52" t="str">
+        <v/>
+      </c>
+      <c r="J52" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="str">
+        <v>MBARGA</v>
+      </c>
+      <c r="B53" t="str">
+        <v>Cécile</v>
+      </c>
+      <c r="C53" t="str">
+        <v>cecile.mbarga.teacher052@edu-nexus.cm</v>
+      </c>
+      <c r="D53" t="str">
+        <v>+237683232441</v>
+      </c>
+      <c r="E53" t="str">
+        <v>ENS-2025-052</v>
+      </c>
+      <c r="F53" t="str">
+        <v>02/10/1992</v>
+      </c>
+      <c r="G53" t="str">
+        <v/>
+      </c>
+      <c r="H53" t="str">
+        <v>Français</v>
+      </c>
+      <c r="I53" t="str">
+        <v/>
+      </c>
+      <c r="J53" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="str">
+        <v>TCHANA</v>
+      </c>
+      <c r="B54" t="str">
+        <v>Armand</v>
+      </c>
+      <c r="C54" t="str">
+        <v>armand.tchana.teacher053@edu-nexus.cm</v>
+      </c>
+      <c r="D54" t="str">
+        <v>+237696570332</v>
+      </c>
+      <c r="E54" t="str">
+        <v>ENS-2025-053</v>
+      </c>
+      <c r="F54" t="str">
+        <v>13/01/1969</v>
+      </c>
+      <c r="G54" t="str">
+        <v/>
+      </c>
+      <c r="H54" t="str">
+        <v>Anglais</v>
+      </c>
+      <c r="I54" t="str">
+        <v/>
+      </c>
+      <c r="J54" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="str">
+        <v>NWANA</v>
+      </c>
+      <c r="B55" t="str">
+        <v>Grace</v>
+      </c>
+      <c r="C55" t="str">
+        <v>grace.nwana.teacher054@edu-nexus.cm</v>
+      </c>
+      <c r="D55" t="str">
+        <v>+237680908223</v>
+      </c>
+      <c r="E55" t="str">
+        <v>ENS-2025-054</v>
+      </c>
+      <c r="F55" t="str">
+        <v>24/04/1976</v>
+      </c>
+      <c r="G55" t="str">
+        <v/>
+      </c>
+      <c r="H55" t="str">
+        <v>Anglais</v>
+      </c>
+      <c r="I55" t="str">
+        <v/>
+      </c>
+      <c r="J55" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="str">
+        <v>MBANGUE</v>
+      </c>
+      <c r="B56" t="str">
+        <v>Lionel</v>
+      </c>
+      <c r="C56" t="str">
+        <v>lionel.mbangue.teacher055@edu-nexus.cm</v>
+      </c>
+      <c r="D56" t="str">
+        <v>+237694246114</v>
+      </c>
+      <c r="E56" t="str">
+        <v>ENS-2025-055</v>
+      </c>
+      <c r="F56" t="str">
+        <v>07/07/1983</v>
+      </c>
+      <c r="G56" t="str">
+        <v/>
+      </c>
+      <c r="H56" t="str">
+        <v>Histoire-Géographie, Histoire, Géographie</v>
+      </c>
+      <c r="I56" t="str">
+        <v/>
+      </c>
+      <c r="J56" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="str">
+        <v>OTTOU</v>
+      </c>
+      <c r="B57" t="str">
+        <v>Francine</v>
+      </c>
+      <c r="C57" t="str">
+        <v>francine.ottou.teacher056@edu-nexus.cm</v>
+      </c>
+      <c r="D57" t="str">
+        <v>+237678584005</v>
+      </c>
+      <c r="E57" t="str">
+        <v>ENS-2025-056</v>
+      </c>
+      <c r="F57" t="str">
+        <v>18/10/1990</v>
+      </c>
+      <c r="G57" t="str">
+        <v/>
+      </c>
+      <c r="H57" t="str">
+        <v>Histoire-Géographie, Histoire, Géographie</v>
+      </c>
+      <c r="I57" t="str">
+        <v/>
+      </c>
+      <c r="J57" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="str">
+        <v>MBIANDA</v>
+      </c>
+      <c r="B58" t="str">
+        <v>Guy</v>
+      </c>
+      <c r="C58" t="str">
+        <v>guy.mbianda.teacher057@edu-nexus.cm</v>
+      </c>
+      <c r="D58" t="str">
+        <v>+237691921896</v>
+      </c>
+      <c r="E58" t="str">
+        <v>ENS-2025-057</v>
+      </c>
+      <c r="F58" t="str">
+        <v>01/01/1967</v>
+      </c>
+      <c r="G58" t="str">
+        <v/>
+      </c>
+      <c r="H58" t="str">
+        <v>Physique-Chimie, Physique, Chimie, Physique-Chimie-Technologie</v>
+      </c>
+      <c r="I58" t="str">
+        <v/>
+      </c>
+      <c r="J58" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="str">
+        <v>NGNOULAYE</v>
+      </c>
+      <c r="B59" t="str">
+        <v>Suzanne</v>
+      </c>
+      <c r="C59" t="str">
+        <v>suzanne.ngnoulaye.teacher058@edu-nexus.cm</v>
+      </c>
+      <c r="D59" t="str">
+        <v>+237676259787</v>
+      </c>
+      <c r="E59" t="str">
+        <v>ENS-2025-058</v>
+      </c>
+      <c r="F59" t="str">
+        <v>12/04/1974</v>
+      </c>
+      <c r="G59" t="str">
+        <v/>
+      </c>
+      <c r="H59" t="str">
+        <v>Sciences, SVT, SVTEEHB</v>
+      </c>
+      <c r="I59" t="str">
+        <v/>
+      </c>
+      <c r="J59" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="str">
+        <v>TSAFACK</v>
+      </c>
+      <c r="B60" t="str">
+        <v>Bruno</v>
+      </c>
+      <c r="C60" t="str">
+        <v>bruno.tsafack.teacher059@edu-nexus.cm</v>
+      </c>
+      <c r="D60" t="str">
+        <v>+237689597678</v>
+      </c>
+      <c r="E60" t="str">
+        <v>ENS-2025-059</v>
+      </c>
+      <c r="F60" t="str">
+        <v>23/07/1981</v>
+      </c>
+      <c r="G60" t="str">
+        <v/>
+      </c>
+      <c r="H60" t="str">
+        <v>EPS</v>
+      </c>
+      <c r="I60" t="str">
+        <v/>
+      </c>
+      <c r="J60" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="str">
+        <v>NDZANA</v>
+      </c>
+      <c r="B61" t="str">
+        <v>Léa</v>
+      </c>
+      <c r="C61" t="str">
+        <v>lea.ndzana.teacher060@edu-nexus.cm</v>
+      </c>
+      <c r="D61" t="str">
+        <v>+237673935569</v>
+      </c>
+      <c r="E61" t="str">
+        <v>ENS-2025-060</v>
+      </c>
+      <c r="F61" t="str">
+        <v>06/10/1988</v>
+      </c>
+      <c r="G61" t="str">
+        <v/>
+      </c>
+      <c r="H61" t="str">
+        <v>EPS</v>
+      </c>
+      <c r="I61" t="str">
+        <v/>
+      </c>
+      <c r="J61" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="str">
+        <v>FOSSO</v>
+      </c>
+      <c r="B62" t="str">
+        <v>Patrick</v>
+      </c>
+      <c r="C62" t="str">
+        <v>patrick.fosso.teacher061@edu-nexus.cm</v>
+      </c>
+      <c r="D62" t="str">
+        <v>+237687273460</v>
+      </c>
+      <c r="E62" t="str">
+        <v>ENS-2025-061</v>
+      </c>
+      <c r="F62" t="str">
+        <v>17/01/1965</v>
+      </c>
+      <c r="G62" t="str">
+        <v/>
+      </c>
+      <c r="H62" t="str">
+        <v>Informatique, Algorithmique-Programmation, Systèmes d'Information</v>
+      </c>
+      <c r="I62" t="str">
+        <v/>
+      </c>
+      <c r="J62" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="str">
+        <v>MBIDA</v>
+      </c>
+      <c r="B63" t="str">
+        <v>Serge</v>
+      </c>
+      <c r="C63" t="str">
+        <v>serge.mbida.teacher062@edu-nexus.cm</v>
+      </c>
+      <c r="D63" t="str">
+        <v>+237671611351</v>
+      </c>
+      <c r="E63" t="str">
+        <v>ENS-2025-062</v>
+      </c>
+      <c r="F63" t="str">
+        <v>28/04/1972</v>
+      </c>
+      <c r="G63" t="str">
+        <v/>
+      </c>
+      <c r="H63" t="str">
+        <v>Lettres classiques (Latin/Grec)</v>
+      </c>
+      <c r="I63" t="str">
+        <v/>
+      </c>
+      <c r="J63" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="str">
+        <v>ONANA</v>
+      </c>
+      <c r="B64" t="str">
+        <v>Véronique</v>
+      </c>
+      <c r="C64" t="str">
+        <v>veronique.onana.teacher063@edu-nexus.cm</v>
+      </c>
+      <c r="D64" t="str">
+        <v>+237684949242</v>
+      </c>
+      <c r="E64" t="str">
+        <v>ENS-2025-063</v>
+      </c>
+      <c r="F64" t="str">
+        <v>11/07/1979</v>
+      </c>
+      <c r="G64" t="str">
+        <v/>
+      </c>
+      <c r="H64" t="str">
+        <v>Lettres classiques (Latin/Grec)</v>
+      </c>
+      <c r="I64" t="str">
+        <v/>
+      </c>
+      <c r="J64" t="str">
         <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:J46"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:J64"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>